<commit_message>
Métricas diarias: ejemplo de 28 días calibrado con los números de los modelos financieros
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/excel/metricas-diarias/01_Metricas_Diarias_Embudo_Low_Ticket.xlsx
+++ b/excel/metricas-diarias/01_Metricas_Diarias_Embudo_Low_Ticket.xlsx
@@ -1257,28 +1257,28 @@
         <v>39488</v>
       </c>
       <c r="F6" s="13" t="n">
-        <v>1450</v>
+        <v>1070</v>
       </c>
       <c r="G6" s="13" t="n">
-        <v>1307</v>
+        <v>965</v>
       </c>
       <c r="H6" s="13" t="n">
-        <v>47</v>
+        <v>34</v>
       </c>
       <c r="I6" s="13" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="J6" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K6" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L6" s="13" t="n">
         <v>1</v>
       </c>
       <c r="M6" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N6" s="13" t="n">
         <v>0</v>
@@ -1405,28 +1405,28 @@
         <v>40565</v>
       </c>
       <c r="F7" s="13" t="n">
-        <v>1317</v>
+        <v>972</v>
       </c>
       <c r="G7" s="13" t="n">
-        <v>1129</v>
+        <v>833</v>
       </c>
       <c r="H7" s="13" t="n">
-        <v>36</v>
+        <v>26</v>
       </c>
       <c r="I7" s="13" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J7" s="13" t="n">
         <v>2</v>
       </c>
       <c r="K7" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L7" s="13" t="n">
         <v>1</v>
       </c>
       <c r="M7" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N7" s="13" t="n">
         <v>0</v>
@@ -1553,25 +1553,25 @@
         <v>47042</v>
       </c>
       <c r="F8" s="13" t="n">
-        <v>1960</v>
+        <v>1447</v>
       </c>
       <c r="G8" s="13" t="n">
-        <v>1829</v>
+        <v>1350</v>
       </c>
       <c r="H8" s="13" t="n">
-        <v>66</v>
+        <v>49</v>
       </c>
       <c r="I8" s="13" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="J8" s="13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K8" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L8" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M8" s="13" t="n">
         <v>1</v>
@@ -1580,7 +1580,7 @@
         <v>0</v>
       </c>
       <c r="O8" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P8" s="13" t="n">
         <v>0</v>
@@ -1701,16 +1701,16 @@
         <v>43811</v>
       </c>
       <c r="F9" s="13" t="n">
-        <v>1219</v>
+        <v>899</v>
       </c>
       <c r="G9" s="13" t="n">
-        <v>1029</v>
+        <v>759</v>
       </c>
       <c r="H9" s="13" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="I9" s="13" t="n">
-        <v>8</v>
+        <v>6</v>
       </c>
       <c r="J9" s="13" t="n">
         <v>2</v>
@@ -1849,19 +1849,19 @@
         <v>40478</v>
       </c>
       <c r="F10" s="13" t="n">
-        <v>1412</v>
+        <v>1042</v>
       </c>
       <c r="G10" s="13" t="n">
-        <v>1271</v>
+        <v>938</v>
       </c>
       <c r="H10" s="13" t="n">
-        <v>46</v>
+        <v>34</v>
       </c>
       <c r="I10" s="13" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J10" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K10" s="13" t="n">
         <v>2</v>
@@ -1997,28 +1997,28 @@
         <v>33742</v>
       </c>
       <c r="F11" s="13" t="n">
-        <v>1372</v>
+        <v>1013</v>
       </c>
       <c r="G11" s="13" t="n">
-        <v>1297</v>
+        <v>957</v>
       </c>
       <c r="H11" s="13" t="n">
-        <v>43</v>
+        <v>32</v>
       </c>
       <c r="I11" s="13" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="J11" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K11" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L11" s="13" t="n">
         <v>1</v>
       </c>
       <c r="M11" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N11" s="13" t="n">
         <v>0</v>
@@ -2145,22 +2145,22 @@
         <v>44418</v>
       </c>
       <c r="F12" s="13" t="n">
-        <v>1550</v>
+        <v>1144</v>
       </c>
       <c r="G12" s="13" t="n">
-        <v>1511</v>
+        <v>1115</v>
       </c>
       <c r="H12" s="13" t="n">
-        <v>51</v>
+        <v>38</v>
       </c>
       <c r="I12" s="13" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="J12" s="13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K12" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L12" s="13" t="n">
         <v>1</v>
@@ -2172,7 +2172,7 @@
         <v>0</v>
       </c>
       <c r="O12" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P12" s="13" t="n">
         <v>0</v>
@@ -2293,31 +2293,31 @@
         <v>59066</v>
       </c>
       <c r="F13" s="13" t="n">
-        <v>2028</v>
+        <v>1497</v>
       </c>
       <c r="G13" s="13" t="n">
-        <v>1812</v>
+        <v>1338</v>
       </c>
       <c r="H13" s="13" t="n">
-        <v>71</v>
+        <v>52</v>
       </c>
       <c r="I13" s="13" t="n">
-        <v>18</v>
+        <v>13</v>
       </c>
       <c r="J13" s="13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K13" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L13" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M13" s="13" t="n">
         <v>1</v>
       </c>
       <c r="N13" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="O13" s="13" t="n">
         <v>1</v>
@@ -2441,28 +2441,28 @@
         <v>36426</v>
       </c>
       <c r="F14" s="13" t="n">
-        <v>1234</v>
+        <v>910</v>
       </c>
       <c r="G14" s="13" t="n">
-        <v>1000</v>
+        <v>738</v>
       </c>
       <c r="H14" s="13" t="n">
-        <v>34</v>
+        <v>25</v>
       </c>
       <c r="I14" s="13" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J14" s="13" t="n">
         <v>2</v>
       </c>
       <c r="K14" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L14" s="13" t="n">
         <v>1</v>
       </c>
       <c r="M14" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N14" s="13" t="n">
         <v>0</v>
@@ -2589,19 +2589,19 @@
         <v>55575</v>
       </c>
       <c r="F15" s="13" t="n">
-        <v>1586</v>
+        <v>1170</v>
       </c>
       <c r="G15" s="13" t="n">
-        <v>1276</v>
+        <v>942</v>
       </c>
       <c r="H15" s="13" t="n">
-        <v>48</v>
+        <v>35</v>
       </c>
       <c r="I15" s="13" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="J15" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K15" s="13" t="n">
         <v>2</v>
@@ -2737,19 +2737,19 @@
         <v>49534</v>
       </c>
       <c r="F16" s="13" t="n">
-        <v>1627</v>
+        <v>1201</v>
       </c>
       <c r="G16" s="13" t="n">
-        <v>1334</v>
+        <v>985</v>
       </c>
       <c r="H16" s="13" t="n">
-        <v>48</v>
+        <v>36</v>
       </c>
       <c r="I16" s="13" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="J16" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K16" s="13" t="n">
         <v>2</v>
@@ -2885,25 +2885,25 @@
         <v>49786</v>
       </c>
       <c r="F17" s="13" t="n">
-        <v>1759</v>
+        <v>1298</v>
       </c>
       <c r="G17" s="13" t="n">
-        <v>1698</v>
+        <v>1254</v>
       </c>
       <c r="H17" s="13" t="n">
-        <v>57</v>
+        <v>42</v>
       </c>
       <c r="I17" s="13" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="J17" s="13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K17" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L17" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M17" s="13" t="n">
         <v>1</v>
@@ -2912,7 +2912,7 @@
         <v>0</v>
       </c>
       <c r="O17" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P17" s="13" t="n">
         <v>0</v>
@@ -3033,19 +3033,19 @@
         <v>39284</v>
       </c>
       <c r="F18" s="13" t="n">
-        <v>1481</v>
+        <v>1093</v>
       </c>
       <c r="G18" s="13" t="n">
-        <v>1205</v>
+        <v>889</v>
       </c>
       <c r="H18" s="13" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="I18" s="13" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="J18" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K18" s="13" t="n">
         <v>2</v>
@@ -3181,28 +3181,28 @@
         <v>41159</v>
       </c>
       <c r="F19" s="13" t="n">
-        <v>1261</v>
+        <v>931</v>
       </c>
       <c r="G19" s="13" t="n">
-        <v>1019</v>
+        <v>752</v>
       </c>
       <c r="H19" s="13" t="n">
-        <v>32</v>
+        <v>24</v>
       </c>
       <c r="I19" s="13" t="n">
-        <v>9</v>
+        <v>6</v>
       </c>
       <c r="J19" s="13" t="n">
         <v>2</v>
       </c>
       <c r="K19" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L19" s="13" t="n">
         <v>1</v>
       </c>
       <c r="M19" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N19" s="13" t="n">
         <v>0</v>
@@ -3329,19 +3329,19 @@
         <v>42195</v>
       </c>
       <c r="F20" s="13" t="n">
-        <v>1359</v>
+        <v>1003</v>
       </c>
       <c r="G20" s="13" t="n">
-        <v>1358</v>
+        <v>1002</v>
       </c>
       <c r="H20" s="13" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="I20" s="13" t="n">
-        <v>13</v>
+        <v>9</v>
       </c>
       <c r="J20" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K20" s="13" t="n">
         <v>2</v>
@@ -3356,7 +3356,7 @@
         <v>0</v>
       </c>
       <c r="O20" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P20" s="13" t="n">
         <v>0</v>
@@ -3477,22 +3477,22 @@
         <v>57331</v>
       </c>
       <c r="F21" s="13" t="n">
-        <v>1940</v>
+        <v>1432</v>
       </c>
       <c r="G21" s="13" t="n">
-        <v>1879</v>
+        <v>1387</v>
       </c>
       <c r="H21" s="13" t="n">
-        <v>62</v>
+        <v>46</v>
       </c>
       <c r="I21" s="13" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="J21" s="13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K21" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L21" s="13" t="n">
         <v>1</v>
@@ -3504,7 +3504,7 @@
         <v>0</v>
       </c>
       <c r="O21" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P21" s="13" t="n">
         <v>0</v>
@@ -3625,22 +3625,22 @@
         <v>46049</v>
       </c>
       <c r="F22" s="13" t="n">
-        <v>1590</v>
+        <v>1173</v>
       </c>
       <c r="G22" s="13" t="n">
-        <v>1562</v>
+        <v>1153</v>
       </c>
       <c r="H22" s="13" t="n">
-        <v>56</v>
+        <v>41</v>
       </c>
       <c r="I22" s="13" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="J22" s="13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K22" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L22" s="13" t="n">
         <v>1</v>
@@ -3652,7 +3652,7 @@
         <v>0</v>
       </c>
       <c r="O22" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P22" s="13" t="n">
         <v>0</v>
@@ -3773,19 +3773,19 @@
         <v>40887</v>
       </c>
       <c r="F23" s="13" t="n">
-        <v>1431</v>
+        <v>1056</v>
       </c>
       <c r="G23" s="13" t="n">
-        <v>1351</v>
+        <v>997</v>
       </c>
       <c r="H23" s="13" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="I23" s="13" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J23" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K23" s="13" t="n">
         <v>2</v>
@@ -3921,19 +3921,19 @@
         <v>52119</v>
       </c>
       <c r="F24" s="13" t="n">
-        <v>1700</v>
+        <v>1255</v>
       </c>
       <c r="G24" s="13" t="n">
-        <v>1372</v>
+        <v>1013</v>
       </c>
       <c r="H24" s="13" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="I24" s="13" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J24" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K24" s="13" t="n">
         <v>2</v>
@@ -4069,28 +4069,28 @@
         <v>49750</v>
       </c>
       <c r="F25" s="13" t="n">
-        <v>1742</v>
+        <v>1286</v>
       </c>
       <c r="G25" s="13" t="n">
-        <v>1456</v>
+        <v>1075</v>
       </c>
       <c r="H25" s="13" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="I25" s="13" t="n">
-        <v>11</v>
+        <v>8</v>
       </c>
       <c r="J25" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K25" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L25" s="13" t="n">
         <v>1</v>
       </c>
       <c r="M25" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N25" s="13" t="n">
         <v>0</v>
@@ -4217,19 +4217,19 @@
         <v>53407</v>
       </c>
       <c r="F26" s="13" t="n">
-        <v>1603</v>
+        <v>1183</v>
       </c>
       <c r="G26" s="13" t="n">
-        <v>1468</v>
+        <v>1083</v>
       </c>
       <c r="H26" s="13" t="n">
-        <v>47</v>
+        <v>35</v>
       </c>
       <c r="I26" s="13" t="n">
-        <v>12</v>
+        <v>9</v>
       </c>
       <c r="J26" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K26" s="13" t="n">
         <v>2</v>
@@ -4365,28 +4365,28 @@
         <v>42193</v>
       </c>
       <c r="F27" s="13" t="n">
-        <v>1539</v>
+        <v>1136</v>
       </c>
       <c r="G27" s="13" t="n">
-        <v>1413</v>
+        <v>1043</v>
       </c>
       <c r="H27" s="13" t="n">
-        <v>45</v>
+        <v>33</v>
       </c>
       <c r="I27" s="13" t="n">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="J27" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K27" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L27" s="13" t="n">
         <v>1</v>
       </c>
       <c r="M27" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N27" s="13" t="n">
         <v>0</v>
@@ -4513,28 +4513,28 @@
         <v>34286</v>
       </c>
       <c r="F28" s="13" t="n">
-        <v>1342</v>
+        <v>990</v>
       </c>
       <c r="G28" s="13" t="n">
-        <v>1069</v>
+        <v>789</v>
       </c>
       <c r="H28" s="13" t="n">
-        <v>39</v>
+        <v>29</v>
       </c>
       <c r="I28" s="13" t="n">
-        <v>10</v>
+        <v>7</v>
       </c>
       <c r="J28" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K28" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="L28" s="13" t="n">
         <v>1</v>
       </c>
       <c r="M28" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="N28" s="13" t="n">
         <v>0</v>
@@ -4661,22 +4661,22 @@
         <v>43982</v>
       </c>
       <c r="F29" s="13" t="n">
-        <v>1486</v>
+        <v>1097</v>
       </c>
       <c r="G29" s="13" t="n">
-        <v>1352</v>
+        <v>998</v>
       </c>
       <c r="H29" s="13" t="n">
-        <v>50</v>
+        <v>37</v>
       </c>
       <c r="I29" s="13" t="n">
-        <v>14</v>
+        <v>11</v>
       </c>
       <c r="J29" s="13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K29" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L29" s="13" t="n">
         <v>1</v>
@@ -4688,7 +4688,7 @@
         <v>0</v>
       </c>
       <c r="O29" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P29" s="13" t="n">
         <v>0</v>
@@ -4809,25 +4809,25 @@
         <v>42026</v>
       </c>
       <c r="F30" s="13" t="n">
-        <v>1662</v>
+        <v>1227</v>
       </c>
       <c r="G30" s="13" t="n">
-        <v>1443</v>
+        <v>1065</v>
       </c>
       <c r="H30" s="13" t="n">
-        <v>53</v>
+        <v>39</v>
       </c>
       <c r="I30" s="13" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="J30" s="13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K30" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L30" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M30" s="13" t="n">
         <v>1</v>
@@ -4836,7 +4836,7 @@
         <v>0</v>
       </c>
       <c r="O30" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P30" s="13" t="n">
         <v>0</v>
@@ -4957,25 +4957,25 @@
         <v>46372</v>
       </c>
       <c r="F31" s="13" t="n">
-        <v>1812</v>
+        <v>1338</v>
       </c>
       <c r="G31" s="13" t="n">
-        <v>1659</v>
+        <v>1225</v>
       </c>
       <c r="H31" s="13" t="n">
-        <v>60</v>
+        <v>44</v>
       </c>
       <c r="I31" s="13" t="n">
-        <v>15</v>
+        <v>11</v>
       </c>
       <c r="J31" s="13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K31" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L31" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M31" s="13" t="n">
         <v>1</v>
@@ -4984,7 +4984,7 @@
         <v>0</v>
       </c>
       <c r="O31" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P31" s="13" t="n">
         <v>0</v>
@@ -5105,25 +5105,25 @@
         <v>49341</v>
       </c>
       <c r="F32" s="13" t="n">
-        <v>1541</v>
+        <v>1137</v>
       </c>
       <c r="G32" s="13" t="n">
-        <v>1551</v>
+        <v>1145</v>
       </c>
       <c r="H32" s="13" t="n">
-        <v>59</v>
+        <v>44</v>
       </c>
       <c r="I32" s="13" t="n">
-        <v>16</v>
+        <v>12</v>
       </c>
       <c r="J32" s="13" t="n">
-        <v>4</v>
+        <v>3</v>
       </c>
       <c r="K32" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="L32" s="13" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="M32" s="13" t="n">
         <v>1</v>
@@ -5132,7 +5132,7 @@
         <v>0</v>
       </c>
       <c r="O32" s="13" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="P32" s="13" t="n">
         <v>0</v>
@@ -5253,19 +5253,19 @@
         <v>40344</v>
       </c>
       <c r="F33" s="13" t="n">
-        <v>1362</v>
+        <v>1005</v>
       </c>
       <c r="G33" s="13" t="n">
-        <v>1326</v>
+        <v>978</v>
       </c>
       <c r="H33" s="13" t="n">
-        <v>42</v>
+        <v>31</v>
       </c>
       <c r="I33" s="13" t="n">
-        <v>12</v>
+        <v>8</v>
       </c>
       <c r="J33" s="13" t="n">
-        <v>3</v>
+        <v>2</v>
       </c>
       <c r="K33" s="13" t="n">
         <v>2</v>

</xml_diff>